<commit_message>
cashop & pvp npc
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B48FB12-1669-4EC6-8ED7-BD77C3DCDD3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E97EFB5-F2BF-43BC-A82F-DCA2742B086A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="276">
   <si>
     <t>string[64]</t>
   </si>
@@ -763,36 +763,6 @@
     <t>iycsa55</t>
   </si>
   <si>
-    <t>ircha01</t>
-  </si>
-  <si>
-    <t>ircha02</t>
-  </si>
-  <si>
-    <t>ircha03</t>
-  </si>
-  <si>
-    <t>ircha04</t>
-  </si>
-  <si>
-    <t>ircha05</t>
-  </si>
-  <si>
-    <t>ircha06</t>
-  </si>
-  <si>
-    <t>ircha07</t>
-  </si>
-  <si>
-    <t>ircha08</t>
-  </si>
-  <si>
-    <t>ircha10</t>
-  </si>
-  <si>
-    <t>ircha11</t>
-  </si>
-  <si>
     <t>ircja09</t>
   </si>
   <si>
@@ -848,6 +818,42 @@
   </si>
   <si>
     <t>ibcsb36</t>
+  </si>
+  <si>
+    <t>ircha13</t>
+  </si>
+  <si>
+    <t>ircha14</t>
+  </si>
+  <si>
+    <t>ircha15</t>
+  </si>
+  <si>
+    <t>ircha16</t>
+  </si>
+  <si>
+    <t>ircha17</t>
+  </si>
+  <si>
+    <t>ircha18</t>
+  </si>
+  <si>
+    <t>ircha19</t>
+  </si>
+  <si>
+    <t>ircha20</t>
+  </si>
+  <si>
+    <t>cash130</t>
+  </si>
+  <si>
+    <t>ircha22</t>
+  </si>
+  <si>
+    <t>ircha23</t>
+  </si>
+  <si>
+    <t>ircha24</t>
   </si>
 </sst>
 </file>
@@ -872,7 +878,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -893,7 +899,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -914,10 +920,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1254,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O131"/>
+  <dimension ref="A1:O132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -1265,8 +1271,7 @@
     <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="14" width="7" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" customWidth="1"/>
-    <col min="18" max="18" width="9.7109375" customWidth="1"/>
+    <col min="17" max="18" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1365,7 +1370,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -1409,7 +1414,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C4">
         <v>150</v>
@@ -1453,7 +1458,7 @@
         <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="C5">
         <v>505</v>
@@ -1497,7 +1502,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -1541,7 +1546,7 @@
         <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C7">
         <v>150</v>
@@ -1585,7 +1590,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="C8">
         <v>505</v>
@@ -1629,7 +1634,7 @@
         <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1673,7 +1678,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C10">
         <v>150</v>
@@ -1717,7 +1722,7 @@
         <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="C11">
         <v>505</v>
@@ -1764,7 +1769,7 @@
         <v>151</v>
       </c>
       <c r="C12">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1808,7 +1813,7 @@
         <v>152</v>
       </c>
       <c r="C13">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1852,7 +1857,7 @@
         <v>153</v>
       </c>
       <c r="C14">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1896,7 +1901,7 @@
         <v>154</v>
       </c>
       <c r="C15">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1940,7 +1945,7 @@
         <v>155</v>
       </c>
       <c r="C16">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1984,7 +1989,7 @@
         <v>156</v>
       </c>
       <c r="C17">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2028,7 +2033,7 @@
         <v>157</v>
       </c>
       <c r="C18">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -2072,7 +2077,7 @@
         <v>158</v>
       </c>
       <c r="C19">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2116,7 +2121,7 @@
         <v>159</v>
       </c>
       <c r="C20">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2160,7 +2165,7 @@
         <v>160</v>
       </c>
       <c r="C21">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -2204,7 +2209,7 @@
         <v>161</v>
       </c>
       <c r="C22">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2248,7 +2253,7 @@
         <v>162</v>
       </c>
       <c r="C23">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2292,7 +2297,7 @@
         <v>163</v>
       </c>
       <c r="C24">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2336,7 +2341,7 @@
         <v>164</v>
       </c>
       <c r="C25">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2380,7 +2385,7 @@
         <v>165</v>
       </c>
       <c r="C26">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2424,7 +2429,7 @@
         <v>166</v>
       </c>
       <c r="C27">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2468,7 +2473,7 @@
         <v>167</v>
       </c>
       <c r="C28">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -2512,7 +2517,7 @@
         <v>168</v>
       </c>
       <c r="C29">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -2556,7 +2561,7 @@
         <v>169</v>
       </c>
       <c r="C30">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -2600,7 +2605,7 @@
         <v>170</v>
       </c>
       <c r="C31">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -2644,7 +2649,7 @@
         <v>171</v>
       </c>
       <c r="C32">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -2688,7 +2693,7 @@
         <v>172</v>
       </c>
       <c r="C33">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -2732,7 +2737,7 @@
         <v>173</v>
       </c>
       <c r="C34">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -2776,7 +2781,7 @@
         <v>174</v>
       </c>
       <c r="C35">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2820,7 +2825,7 @@
         <v>175</v>
       </c>
       <c r="C36">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -2864,7 +2869,7 @@
         <v>176</v>
       </c>
       <c r="C37">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -2908,7 +2913,7 @@
         <v>177</v>
       </c>
       <c r="C38">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -2952,7 +2957,7 @@
         <v>178</v>
       </c>
       <c r="C39">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -2996,7 +3001,7 @@
         <v>179</v>
       </c>
       <c r="C40">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -3033,14 +3038,14 @@
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
+      <c r="A41" t="s">
         <v>59</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="C41">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -3077,14 +3082,14 @@
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
+      <c r="A42" t="s">
         <v>60</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C42">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -3121,14 +3126,14 @@
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
+      <c r="A43" t="s">
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="C43">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -3165,14 +3170,14 @@
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
+      <c r="A44" t="s">
         <v>62</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="C44">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -3209,14 +3214,14 @@
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
+      <c r="A45" t="s">
         <v>63</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C45">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -3253,14 +3258,14 @@
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
+      <c r="A46" t="s">
         <v>64</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="C46">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -3297,14 +3302,14 @@
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
+      <c r="A47" t="s">
         <v>65</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C47">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -3341,14 +3346,14 @@
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
+      <c r="A48" t="s">
         <v>66</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="C48">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -3385,14 +3390,14 @@
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
+      <c r="A49" t="s">
         <v>67</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="C49">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -3429,14 +3434,14 @@
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
+      <c r="A50" t="s">
         <v>68</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="C50">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -3480,7 +3485,7 @@
         <v>180</v>
       </c>
       <c r="C51">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -3524,7 +3529,7 @@
         <v>181</v>
       </c>
       <c r="C52">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -3568,7 +3573,7 @@
         <v>182</v>
       </c>
       <c r="C53">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -3612,7 +3617,7 @@
         <v>183</v>
       </c>
       <c r="C54">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -3656,7 +3661,7 @@
         <v>184</v>
       </c>
       <c r="C55">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -3700,7 +3705,7 @@
         <v>185</v>
       </c>
       <c r="C56">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -3744,7 +3749,7 @@
         <v>186</v>
       </c>
       <c r="C57">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -3788,7 +3793,7 @@
         <v>187</v>
       </c>
       <c r="C58">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -3832,7 +3837,7 @@
         <v>188</v>
       </c>
       <c r="C59">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -3876,7 +3881,7 @@
         <v>189</v>
       </c>
       <c r="C60">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -3920,7 +3925,7 @@
         <v>190</v>
       </c>
       <c r="C61">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -3964,7 +3969,7 @@
         <v>191</v>
       </c>
       <c r="C62">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -4008,7 +4013,7 @@
         <v>192</v>
       </c>
       <c r="C63">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -4052,7 +4057,7 @@
         <v>193</v>
       </c>
       <c r="C64">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -4096,7 +4101,7 @@
         <v>194</v>
       </c>
       <c r="C65">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -4140,7 +4145,7 @@
         <v>195</v>
       </c>
       <c r="C66">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D66">
         <v>1</v>
@@ -4184,7 +4189,7 @@
         <v>196</v>
       </c>
       <c r="C67">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D67">
         <v>1</v>
@@ -4228,7 +4233,7 @@
         <v>197</v>
       </c>
       <c r="C68">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="D68">
         <v>1</v>
@@ -4932,7 +4937,7 @@
         <v>213</v>
       </c>
       <c r="C84">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D84">
         <v>1</v>
@@ -6204,8 +6209,8 @@
       <c r="A113" t="s">
         <v>132</v>
       </c>
-      <c r="B113" s="2" t="s">
-        <v>245</v>
+      <c r="B113" s="3" t="s">
+        <v>264</v>
       </c>
       <c r="C113">
         <v>20</v>
@@ -6248,8 +6253,8 @@
       <c r="A114" t="s">
         <v>133</v>
       </c>
-      <c r="B114" s="2" t="s">
-        <v>246</v>
+      <c r="B114" s="3" t="s">
+        <v>265</v>
       </c>
       <c r="C114">
         <v>20</v>
@@ -6292,8 +6297,8 @@
       <c r="A115" t="s">
         <v>134</v>
       </c>
-      <c r="B115" s="2" t="s">
-        <v>247</v>
+      <c r="B115" s="3" t="s">
+        <v>266</v>
       </c>
       <c r="C115">
         <v>20</v>
@@ -6336,8 +6341,8 @@
       <c r="A116" t="s">
         <v>135</v>
       </c>
-      <c r="B116" s="2" t="s">
-        <v>248</v>
+      <c r="B116" s="3" t="s">
+        <v>267</v>
       </c>
       <c r="C116">
         <v>20</v>
@@ -6380,8 +6385,8 @@
       <c r="A117" t="s">
         <v>136</v>
       </c>
-      <c r="B117" s="2" t="s">
-        <v>249</v>
+      <c r="B117" s="3" t="s">
+        <v>268</v>
       </c>
       <c r="C117">
         <v>20</v>
@@ -6424,8 +6429,8 @@
       <c r="A118" t="s">
         <v>137</v>
       </c>
-      <c r="B118" s="2" t="s">
-        <v>250</v>
+      <c r="B118" s="3" t="s">
+        <v>269</v>
       </c>
       <c r="C118">
         <v>20</v>
@@ -6468,8 +6473,8 @@
       <c r="A119" t="s">
         <v>138</v>
       </c>
-      <c r="B119" s="2" t="s">
-        <v>251</v>
+      <c r="B119" s="3" t="s">
+        <v>270</v>
       </c>
       <c r="C119">
         <v>20</v>
@@ -6512,8 +6517,8 @@
       <c r="A120" t="s">
         <v>139</v>
       </c>
-      <c r="B120" s="2" t="s">
-        <v>252</v>
+      <c r="B120" s="3" t="s">
+        <v>271</v>
       </c>
       <c r="C120">
         <v>20</v>
@@ -6556,8 +6561,8 @@
       <c r="A121" t="s">
         <v>140</v>
       </c>
-      <c r="B121" s="2" t="s">
-        <v>253</v>
+      <c r="B121" s="3" t="s">
+        <v>273</v>
       </c>
       <c r="C121">
         <v>20</v>
@@ -6600,8 +6605,8 @@
       <c r="A122" t="s">
         <v>141</v>
       </c>
-      <c r="B122" s="2" t="s">
-        <v>254</v>
+      <c r="B122" s="3" t="s">
+        <v>274</v>
       </c>
       <c r="C122">
         <v>20</v>
@@ -6644,11 +6649,11 @@
       <c r="A123" t="s">
         <v>142</v>
       </c>
-      <c r="B123" s="2" t="s">
-        <v>260</v>
+      <c r="B123" s="3" t="s">
+        <v>275</v>
       </c>
       <c r="C123">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -6689,10 +6694,10 @@
         <v>143</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="C124">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -6733,10 +6738,10 @@
         <v>144</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C125">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -6777,10 +6782,10 @@
         <v>145</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="C126">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -6821,10 +6826,10 @@
         <v>146</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C127">
-        <v>105</v>
+        <v>250</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -6865,10 +6870,10 @@
         <v>147</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="C128">
-        <v>305</v>
+        <v>105</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -6909,10 +6914,10 @@
         <v>148</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="C129">
-        <v>505</v>
+        <v>305</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -6953,10 +6958,10 @@
         <v>149</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="C130">
-        <v>1005</v>
+        <v>505</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -6997,42 +7002,86 @@
         <v>150</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="C131">
+        <v>1005</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F131">
+        <v>-1</v>
+      </c>
+      <c r="G131">
+        <v>0</v>
+      </c>
+      <c r="H131">
+        <v>0</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>0</v>
+      </c>
+      <c r="L131">
+        <v>0</v>
+      </c>
+      <c r="M131">
+        <v>0</v>
+      </c>
+      <c r="N131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>272</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C132">
         <v>150</v>
       </c>
-      <c r="D131">
-        <v>1</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F131">
-        <v>-1</v>
-      </c>
-      <c r="G131">
-        <v>0</v>
-      </c>
-      <c r="H131">
-        <v>0</v>
-      </c>
-      <c r="I131">
-        <v>0</v>
-      </c>
-      <c r="J131">
-        <v>0</v>
-      </c>
-      <c r="K131">
-        <v>0</v>
-      </c>
-      <c r="L131">
-        <v>0</v>
-      </c>
-      <c r="M131">
-        <v>0</v>
-      </c>
-      <c r="N131">
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F132">
+        <v>-1</v>
+      </c>
+      <c r="G132">
+        <v>0</v>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>0</v>
+      </c>
+      <c r="L132">
+        <v>0</v>
+      </c>
+      <c r="M132">
+        <v>0</v>
+      </c>
+      <c r="N132">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
crit & smart potion price fix
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E97EFB5-F2BF-43BC-A82F-DCA2742B086A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B04DF5-1582-4588-BEEA-95FF83DB57F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4321,7 +4321,7 @@
         <v>199</v>
       </c>
       <c r="C70">
-        <v>210</v>
+        <v>2</v>
       </c>
       <c r="D70">
         <v>1</v>
@@ -4365,7 +4365,7 @@
         <v>200</v>
       </c>
       <c r="C71">
-        <v>211</v>
+        <v>2</v>
       </c>
       <c r="D71">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         <v>202</v>
       </c>
       <c r="C73">
-        <v>213</v>
+        <v>2</v>
       </c>
       <c r="D73">
         <v>1</v>
@@ -4497,7 +4497,7 @@
         <v>203</v>
       </c>
       <c r="C74">
-        <v>214</v>
+        <v>2</v>
       </c>
       <c r="D74">
         <v>1</v>

</xml_diff>

<commit_message>
broadcast add on cashop
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B04DF5-1582-4588-BEEA-95FF83DB57F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C04237B3-79D0-4EE1-96B4-142083D02E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="279">
   <si>
     <t>string[64]</t>
   </si>
@@ -854,6 +854,15 @@
   </si>
   <si>
     <t>ircha24</t>
+  </si>
+  <si>
+    <t>cash131</t>
+  </si>
+  <si>
+    <t>iybrd01</t>
+  </si>
+  <si>
+    <t>ne/be/0/0/0</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1269,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O132"/>
+  <dimension ref="A1:O133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -7085,6 +7094,50 @@
         <v>0</v>
       </c>
     </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>276</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C133">
+        <v>5</v>
+      </c>
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F133">
+        <v>-1</v>
+      </c>
+      <c r="G133">
+        <v>0</v>
+      </c>
+      <c r="H133">
+        <v>0</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>0</v>
+      </c>
+      <c r="L133">
+        <v>0</v>
+      </c>
+      <c r="M133">
+        <v>0</v>
+      </c>
+      <c r="N133">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ADD PREMIUM CURE POTS 1.5 SEC IN CASH SHOP AND PRICE IN 5 CC EACH
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5614D9AE-E9C7-4AAF-964F-2013B065B504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DFF500-58AD-4B7B-9E66-ACD76B5206EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="285">
   <si>
     <t>string[64]</t>
   </si>
@@ -863,6 +863,24 @@
   </si>
   <si>
     <t>ne/be/0/0/0</t>
+  </si>
+  <si>
+    <t>cash132</t>
+  </si>
+  <si>
+    <t>cash133</t>
+  </si>
+  <si>
+    <t>cash134</t>
+  </si>
+  <si>
+    <t>ipcsa34</t>
+  </si>
+  <si>
+    <t>ipcsa35</t>
+  </si>
+  <si>
+    <t>ipcsa36</t>
   </si>
 </sst>
 </file>
@@ -1269,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O133"/>
+  <dimension ref="A1:O136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -7094,7 +7112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>276</v>
       </c>
@@ -7135,6 +7153,138 @@
         <v>0</v>
       </c>
       <c r="N133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>279</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C134">
+        <v>5</v>
+      </c>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F134">
+        <v>-1</v>
+      </c>
+      <c r="G134">
+        <v>0</v>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0</v>
+      </c>
+      <c r="L134">
+        <v>0</v>
+      </c>
+      <c r="M134">
+        <v>0</v>
+      </c>
+      <c r="N134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>280</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C135">
+        <v>5</v>
+      </c>
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F135">
+        <v>-1</v>
+      </c>
+      <c r="G135">
+        <v>0</v>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>0</v>
+      </c>
+      <c r="L135">
+        <v>0</v>
+      </c>
+      <c r="M135">
+        <v>0</v>
+      </c>
+      <c r="N135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>281</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C136">
+        <v>5</v>
+      </c>
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F136">
+        <v>-1</v>
+      </c>
+      <c r="G136">
+        <v>0</v>
+      </c>
+      <c r="H136">
+        <v>0</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+      <c r="L136">
+        <v>0</v>
+      </c>
+      <c r="M136">
+        <v>0</v>
+      </c>
+      <c r="N136">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
supper smart & crit potion cashop price fix
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DFF500-58AD-4B7B-9E66-ACD76B5206EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1383306-5313-4B0D-BD6C-8FFA8D7847FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4304,7 +4304,7 @@
         <v>198</v>
       </c>
       <c r="C69">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D69">
         <v>1</v>
@@ -4348,7 +4348,7 @@
         <v>199</v>
       </c>
       <c r="C70">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D70">
         <v>1</v>
@@ -4392,7 +4392,7 @@
         <v>200</v>
       </c>
       <c r="C71">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D71">
         <v>1</v>
@@ -4436,7 +4436,7 @@
         <v>201</v>
       </c>
       <c r="C72">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D72">
         <v>1</v>
@@ -4480,7 +4480,7 @@
         <v>202</v>
       </c>
       <c r="C73">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D73">
         <v>1</v>
@@ -4524,7 +4524,7 @@
         <v>203</v>
       </c>
       <c r="C74">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D74">
         <v>1</v>
@@ -5668,7 +5668,7 @@
         <v>232</v>
       </c>
       <c r="C100">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D100">
         <v>1</v>
@@ -5712,7 +5712,7 @@
         <v>233</v>
       </c>
       <c r="C101">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D101">
         <v>1</v>
@@ -5756,7 +5756,7 @@
         <v>234</v>
       </c>
       <c r="C102">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D102">
         <v>1</v>
@@ -5932,7 +5932,7 @@
         <v>238</v>
       </c>
       <c r="C106">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -5976,7 +5976,7 @@
         <v>239</v>
       </c>
       <c r="C107">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -6020,7 +6020,7 @@
         <v>240</v>
       </c>
       <c r="C108">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D108">
         <v>1</v>

</xml_diff>

<commit_message>
ADD ALL AMMO EXPLODING BEAM IN CASH SHOP SAME  PRICE
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1383306-5313-4B0D-BD6C-8FFA8D7847FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5465A3C4-3B52-4088-BFDD-DA7FB71348A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="295">
   <si>
     <t>string[64]</t>
   </si>
@@ -881,6 +881,36 @@
   </si>
   <si>
     <t>ipcsa36</t>
+  </si>
+  <si>
+    <t>cash135</t>
+  </si>
+  <si>
+    <t>cash136</t>
+  </si>
+  <si>
+    <t>cash137</t>
+  </si>
+  <si>
+    <t>cash138</t>
+  </si>
+  <si>
+    <t>cash139</t>
+  </si>
+  <si>
+    <t>ibcsb37</t>
+  </si>
+  <si>
+    <t>ibcsb38</t>
+  </si>
+  <si>
+    <t>ibcsb39</t>
+  </si>
+  <si>
+    <t>ibcsb40</t>
+  </si>
+  <si>
+    <t>ibcsb41</t>
   </si>
 </sst>
 </file>
@@ -1287,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O136"/>
+  <dimension ref="A1:O141"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -7288,6 +7318,226 @@
         <v>0</v>
       </c>
     </row>
+    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>285</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C137">
+        <v>100</v>
+      </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F137">
+        <v>-1</v>
+      </c>
+      <c r="G137">
+        <v>0</v>
+      </c>
+      <c r="H137">
+        <v>1</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>0</v>
+      </c>
+      <c r="L137">
+        <v>0</v>
+      </c>
+      <c r="M137">
+        <v>0</v>
+      </c>
+      <c r="N137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>286</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C138">
+        <v>100</v>
+      </c>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F138">
+        <v>-1</v>
+      </c>
+      <c r="G138">
+        <v>0</v>
+      </c>
+      <c r="H138">
+        <v>1</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0</v>
+      </c>
+      <c r="L138">
+        <v>0</v>
+      </c>
+      <c r="M138">
+        <v>0</v>
+      </c>
+      <c r="N138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>287</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C139">
+        <v>100</v>
+      </c>
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F139">
+        <v>-1</v>
+      </c>
+      <c r="G139">
+        <v>0</v>
+      </c>
+      <c r="H139">
+        <v>1</v>
+      </c>
+      <c r="I139">
+        <v>0</v>
+      </c>
+      <c r="J139">
+        <v>0</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
+      <c r="L139">
+        <v>0</v>
+      </c>
+      <c r="M139">
+        <v>0</v>
+      </c>
+      <c r="N139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>288</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C140">
+        <v>100</v>
+      </c>
+      <c r="D140">
+        <v>1</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F140">
+        <v>-1</v>
+      </c>
+      <c r="G140">
+        <v>0</v>
+      </c>
+      <c r="H140">
+        <v>1</v>
+      </c>
+      <c r="I140">
+        <v>0</v>
+      </c>
+      <c r="J140">
+        <v>0</v>
+      </c>
+      <c r="K140">
+        <v>0</v>
+      </c>
+      <c r="L140">
+        <v>0</v>
+      </c>
+      <c r="M140">
+        <v>0</v>
+      </c>
+      <c r="N140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>289</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C141">
+        <v>100</v>
+      </c>
+      <c r="D141">
+        <v>1</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F141">
+        <v>-1</v>
+      </c>
+      <c r="G141">
+        <v>0</v>
+      </c>
+      <c r="H141">
+        <v>1</v>
+      </c>
+      <c r="I141">
+        <v>0</v>
+      </c>
+      <c r="J141">
+        <v>0</v>
+      </c>
+      <c r="K141">
+        <v>0</v>
+      </c>
+      <c r="L141">
+        <v>0</v>
+      </c>
+      <c r="M141">
+        <v>0</v>
+      </c>
+      <c r="N141">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
cashop potato, hot choco, wing prototype price all race
</commit_message>
<xml_diff>
--- a/gu_in/ItemCash.edf/CashShop.xlsx
+++ b/gu_in/ItemCash.edf/CashShop.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3AA848-26DA-4A36-AA62-9B4416800238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962A2B1A-942B-43C4-9098-E288A48BFEFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5970" yWindow="705" windowWidth="17565" windowHeight="11205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CashShop" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="291">
   <si>
     <t>string[64]</t>
   </si>
@@ -640,12 +640,6 @@
     <t>ipcsb10</t>
   </si>
   <si>
-    <t>ipevn07</t>
-  </si>
-  <si>
-    <t>ipevn06</t>
-  </si>
-  <si>
     <t>ipdou01</t>
   </si>
   <si>
@@ -890,12 +884,6 @@
   </si>
   <si>
     <t>cash137</t>
-  </si>
-  <si>
-    <t>cash138</t>
-  </si>
-  <si>
-    <t>cash139</t>
   </si>
   <si>
     <t>ibcsb42</t>
@@ -1317,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O141"/>
+  <dimension ref="A1:O139"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -1427,7 +1415,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -1445,7 +1433,7 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1471,7 +1459,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C4">
         <v>150</v>
@@ -1489,7 +1477,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1515,7 +1503,7 @@
         <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C5">
         <v>505</v>
@@ -1559,7 +1547,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -1577,7 +1565,7 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1603,7 +1591,7 @@
         <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C7">
         <v>150</v>
@@ -1621,7 +1609,7 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1647,7 +1635,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C8">
         <v>505</v>
@@ -1691,7 +1679,7 @@
         <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1709,7 +1697,7 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1735,7 +1723,7 @@
         <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C10">
         <v>150</v>
@@ -1753,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1779,7 +1767,7 @@
         <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C11">
         <v>505</v>
@@ -1841,7 +1829,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -1885,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1929,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1973,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -2017,7 +2005,7 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -2061,7 +2049,7 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17">
         <v>0</v>
@@ -2105,7 +2093,7 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -2149,7 +2137,7 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -2193,7 +2181,7 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -2237,7 +2225,7 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -2281,7 +2269,7 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -2325,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -2369,7 +2357,7 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -2413,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -2457,7 +2445,7 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -2501,7 +2489,7 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -2545,7 +2533,7 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -2589,7 +2577,7 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -2633,7 +2621,7 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -2677,7 +2665,7 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -2721,7 +2709,7 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -2765,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -2809,7 +2797,7 @@
         <v>0</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -2853,7 +2841,7 @@
         <v>0</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -2897,7 +2885,7 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -2941,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="H37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -2985,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="H38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I38">
         <v>0</v>
@@ -3029,7 +3017,7 @@
         <v>0</v>
       </c>
       <c r="H39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -3073,7 +3061,7 @@
         <v>0</v>
       </c>
       <c r="H40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -3099,7 +3087,7 @@
         <v>59</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -3117,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -3143,7 +3131,7 @@
         <v>60</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C42">
         <v>100</v>
@@ -3161,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42">
         <v>0</v>
@@ -3187,7 +3175,7 @@
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -3205,7 +3193,7 @@
         <v>0</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -3231,7 +3219,7 @@
         <v>62</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -3249,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="H44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -3275,7 +3263,7 @@
         <v>63</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C45">
         <v>100</v>
@@ -3293,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="H45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I45">
         <v>0</v>
@@ -3319,7 +3307,7 @@
         <v>64</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -3337,7 +3325,7 @@
         <v>0</v>
       </c>
       <c r="H46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46">
         <v>0</v>
@@ -3363,7 +3351,7 @@
         <v>65</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -3381,7 +3369,7 @@
         <v>0</v>
       </c>
       <c r="H47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -3407,7 +3395,7 @@
         <v>66</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -3425,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I48">
         <v>0</v>
@@ -3451,7 +3439,7 @@
         <v>67</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C49">
         <v>100</v>
@@ -3469,7 +3457,7 @@
         <v>0</v>
       </c>
       <c r="H49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I49">
         <v>0</v>
@@ -3495,7 +3483,7 @@
         <v>68</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C50">
         <v>100</v>
@@ -3513,7 +3501,7 @@
         <v>0</v>
       </c>
       <c r="H50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50">
         <v>0</v>
@@ -4349,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="H69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I69">
         <v>0</v>
@@ -4393,7 +4381,7 @@
         <v>0</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I70">
         <v>0</v>
@@ -4437,7 +4425,7 @@
         <v>0</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I71">
         <v>0</v>
@@ -4481,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="H72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I72">
         <v>0</v>
@@ -4525,7 +4513,7 @@
         <v>0</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I73">
         <v>0</v>
@@ -4569,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I74">
         <v>0</v>
@@ -4598,7 +4586,7 @@
         <v>204</v>
       </c>
       <c r="C75">
-        <v>10</v>
+        <v>300</v>
       </c>
       <c r="D75">
         <v>1</v>
@@ -4607,7 +4595,7 @@
         <v>18</v>
       </c>
       <c r="F75">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G75">
         <v>0</v>
@@ -4642,7 +4630,7 @@
         <v>205</v>
       </c>
       <c r="C76">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D76">
         <v>1</v>
@@ -4686,7 +4674,7 @@
         <v>206</v>
       </c>
       <c r="C77">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D77">
         <v>1</v>
@@ -4695,7 +4683,7 @@
         <v>18</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G77">
         <v>0</v>
@@ -4730,7 +4718,7 @@
         <v>207</v>
       </c>
       <c r="C78">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D78">
         <v>1</v>
@@ -4774,7 +4762,7 @@
         <v>208</v>
       </c>
       <c r="C79">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D79">
         <v>1</v>
@@ -4818,7 +4806,7 @@
         <v>209</v>
       </c>
       <c r="C80">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D80">
         <v>1</v>
@@ -4862,7 +4850,7 @@
         <v>210</v>
       </c>
       <c r="C81">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D81">
         <v>1</v>
@@ -4912,7 +4900,7 @@
         <v>1</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F82">
         <v>-1</v>
@@ -4947,16 +4935,16 @@
         <v>101</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C83">
+        <v>10</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C83">
-        <v>300</v>
-      </c>
-      <c r="D83">
-        <v>1</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="F83">
         <v>-1</v>
@@ -4991,16 +4979,16 @@
         <v>102</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C84">
-        <v>300</v>
+        <v>10</v>
       </c>
       <c r="D84">
         <v>1</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F84">
         <v>-1</v>
@@ -5030,7 +5018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>103</v>
       </c>
@@ -5038,13 +5026,13 @@
         <v>215</v>
       </c>
       <c r="C85">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="D85">
         <v>1</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>214</v>
+        <v>22</v>
       </c>
       <c r="F85">
         <v>-1</v>
@@ -5053,7 +5041,7 @@
         <v>0</v>
       </c>
       <c r="H85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I85">
         <v>0</v>
@@ -5082,13 +5070,13 @@
         <v>216</v>
       </c>
       <c r="C86">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D86">
         <v>1</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F86">
         <v>-1</v>
@@ -5097,7 +5085,7 @@
         <v>0</v>
       </c>
       <c r="H86">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I86">
         <v>0</v>
@@ -5118,7 +5106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>105</v>
       </c>
@@ -5126,13 +5114,13 @@
         <v>217</v>
       </c>
       <c r="C87">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="D87">
         <v>1</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F87">
         <v>-1</v>
@@ -5185,7 +5173,7 @@
         <v>0</v>
       </c>
       <c r="H88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I88">
         <v>0</v>
@@ -5211,7 +5199,7 @@
         <v>107</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C89">
         <v>2</v>
@@ -5220,7 +5208,7 @@
         <v>1</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>30</v>
+        <v>221</v>
       </c>
       <c r="F89">
         <v>-1</v>
@@ -5229,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="H89">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I89">
         <v>0</v>
@@ -5255,7 +5243,7 @@
         <v>108</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C90">
         <v>2</v>
@@ -5264,7 +5252,7 @@
         <v>1</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>30</v>
+        <v>221</v>
       </c>
       <c r="F90">
         <v>-1</v>
@@ -5273,7 +5261,7 @@
         <v>0</v>
       </c>
       <c r="H90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I90">
         <v>0</v>
@@ -5299,7 +5287,7 @@
         <v>109</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C91">
         <v>2</v>
@@ -5308,7 +5296,7 @@
         <v>1</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F91">
         <v>-1</v>
@@ -5317,7 +5305,7 @@
         <v>0</v>
       </c>
       <c r="H91">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I91">
         <v>0</v>
@@ -5352,7 +5340,7 @@
         <v>1</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>223</v>
+        <v>118</v>
       </c>
       <c r="F92">
         <v>-1</v>
@@ -5361,7 +5349,7 @@
         <v>0</v>
       </c>
       <c r="H92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I92">
         <v>0</v>
@@ -5396,7 +5384,7 @@
         <v>1</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>223</v>
+        <v>118</v>
       </c>
       <c r="F93">
         <v>-1</v>
@@ -5405,7 +5393,7 @@
         <v>0</v>
       </c>
       <c r="H93">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I93">
         <v>0</v>
@@ -5449,7 +5437,7 @@
         <v>0</v>
       </c>
       <c r="H94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I94">
         <v>0</v>
@@ -5484,7 +5472,7 @@
         <v>1</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>118</v>
+        <v>219</v>
       </c>
       <c r="F95">
         <v>-1</v>
@@ -5493,7 +5481,7 @@
         <v>0</v>
       </c>
       <c r="H95">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I95">
         <v>0</v>
@@ -5528,7 +5516,7 @@
         <v>1</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>118</v>
+        <v>219</v>
       </c>
       <c r="F96">
         <v>-1</v>
@@ -5537,7 +5525,7 @@
         <v>0</v>
       </c>
       <c r="H96">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I96">
         <v>0</v>
@@ -5572,7 +5560,7 @@
         <v>1</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F97">
         <v>-1</v>
@@ -5581,7 +5569,7 @@
         <v>0</v>
       </c>
       <c r="H97">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -5616,7 +5604,7 @@
         <v>1</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F98">
         <v>-1</v>
@@ -5625,7 +5613,7 @@
         <v>0</v>
       </c>
       <c r="H98">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I98">
         <v>0</v>
@@ -5660,7 +5648,7 @@
         <v>1</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F99">
         <v>-1</v>
@@ -5669,7 +5657,7 @@
         <v>0</v>
       </c>
       <c r="H99">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I99">
         <v>0</v>
@@ -5704,7 +5692,7 @@
         <v>1</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F100">
         <v>-1</v>
@@ -5713,7 +5701,7 @@
         <v>0</v>
       </c>
       <c r="H100">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I100">
         <v>0</v>
@@ -5742,13 +5730,13 @@
         <v>233</v>
       </c>
       <c r="C101">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D101">
         <v>1</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>221</v>
+        <v>30</v>
       </c>
       <c r="F101">
         <v>-1</v>
@@ -5757,7 +5745,7 @@
         <v>0</v>
       </c>
       <c r="H101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I101">
         <v>0</v>
@@ -5786,13 +5774,13 @@
         <v>234</v>
       </c>
       <c r="C102">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D102">
         <v>1</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>221</v>
+        <v>30</v>
       </c>
       <c r="F102">
         <v>-1</v>
@@ -5801,7 +5789,7 @@
         <v>0</v>
       </c>
       <c r="H102">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I102">
         <v>0</v>
@@ -5845,7 +5833,7 @@
         <v>0</v>
       </c>
       <c r="H103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I103">
         <v>0</v>
@@ -5874,13 +5862,13 @@
         <v>236</v>
       </c>
       <c r="C104">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D104">
         <v>1</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="F104">
         <v>-1</v>
@@ -5889,7 +5877,7 @@
         <v>0</v>
       </c>
       <c r="H104">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I104">
         <v>0</v>
@@ -5918,13 +5906,13 @@
         <v>237</v>
       </c>
       <c r="C105">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D105">
         <v>1</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="F105">
         <v>-1</v>
@@ -5933,7 +5921,7 @@
         <v>0</v>
       </c>
       <c r="H105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I105">
         <v>0</v>
@@ -5977,7 +5965,7 @@
         <v>0</v>
       </c>
       <c r="H106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I106">
         <v>0</v>
@@ -6006,13 +5994,13 @@
         <v>239</v>
       </c>
       <c r="C107">
-        <v>2</v>
+        <v>500</v>
       </c>
       <c r="D107">
         <v>1</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="F107">
         <v>-1</v>
@@ -6021,7 +6009,7 @@
         <v>0</v>
       </c>
       <c r="H107">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I107">
         <v>0</v>
@@ -6050,13 +6038,13 @@
         <v>240</v>
       </c>
       <c r="C108">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="D108">
         <v>1</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>118</v>
+        <v>20</v>
       </c>
       <c r="F108">
         <v>-1</v>
@@ -6065,7 +6053,7 @@
         <v>0</v>
       </c>
       <c r="H108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I108">
         <v>0</v>
@@ -6094,13 +6082,13 @@
         <v>241</v>
       </c>
       <c r="C109">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="D109">
         <v>1</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F109">
         <v>-1</v>
@@ -6178,17 +6166,17 @@
       <c r="A111" t="s">
         <v>130</v>
       </c>
-      <c r="B111" s="2" t="s">
-        <v>243</v>
+      <c r="B111" s="3" t="s">
+        <v>262</v>
       </c>
       <c r="C111">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F111">
         <v>-1</v>
@@ -6222,17 +6210,17 @@
       <c r="A112" t="s">
         <v>131</v>
       </c>
-      <c r="B112" s="2" t="s">
-        <v>244</v>
+      <c r="B112" s="3" t="s">
+        <v>263</v>
       </c>
       <c r="C112">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D112">
         <v>1</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F112">
         <v>-1</v>
@@ -6531,7 +6519,7 @@
         <v>138</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C119">
         <v>60</v>
@@ -6575,7 +6563,7 @@
         <v>139</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C120">
         <v>60</v>
@@ -6662,11 +6650,11 @@
       <c r="A122" t="s">
         <v>141</v>
       </c>
-      <c r="B122" s="3" t="s">
-        <v>274</v>
+      <c r="B122" s="2" t="s">
+        <v>248</v>
       </c>
       <c r="C122">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -6706,11 +6694,11 @@
       <c r="A123" t="s">
         <v>142</v>
       </c>
-      <c r="B123" s="3" t="s">
-        <v>275</v>
+      <c r="B123" s="2" t="s">
+        <v>249</v>
       </c>
       <c r="C123">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -6754,7 +6742,7 @@
         <v>250</v>
       </c>
       <c r="C124">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -6798,7 +6786,7 @@
         <v>251</v>
       </c>
       <c r="C125">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -6839,10 +6827,10 @@
         <v>145</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C126">
-        <v>150</v>
+        <v>105</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -6883,10 +6871,10 @@
         <v>146</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C127">
-        <v>250</v>
+        <v>305</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -6930,7 +6918,7 @@
         <v>247</v>
       </c>
       <c r="C128">
-        <v>105</v>
+        <v>505</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -6971,10 +6959,10 @@
         <v>148</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C129">
-        <v>305</v>
+        <v>1005</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -7015,10 +7003,10 @@
         <v>149</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C130">
-        <v>505</v>
+        <v>150</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -7054,21 +7042,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>150</v>
       </c>
-      <c r="B131" s="2" t="s">
-        <v>246</v>
+      <c r="B131" s="3" t="s">
+        <v>275</v>
       </c>
       <c r="C131">
-        <v>1005</v>
+        <v>5</v>
       </c>
       <c r="D131">
         <v>1</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>18</v>
+        <v>276</v>
       </c>
       <c r="F131">
         <v>-1</v>
@@ -7100,19 +7088,19 @@
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>272</v>
-      </c>
-      <c r="B132" s="2" t="s">
-        <v>245</v>
+        <v>270</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>280</v>
       </c>
       <c r="C132">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="D132">
         <v>1</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>18</v>
+        <v>276</v>
       </c>
       <c r="F132">
         <v>-1</v>
@@ -7142,12 +7130,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C133">
         <v>5</v>
@@ -7156,7 +7144,7 @@
         <v>1</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F133">
         <v>-1</v>
@@ -7188,7 +7176,7 @@
     </row>
     <row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>282</v>
@@ -7200,7 +7188,7 @@
         <v>1</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F134">
         <v>-1</v>
@@ -7232,19 +7220,19 @@
     </row>
     <row r="135" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>280</v>
-      </c>
-      <c r="B135" s="3" t="s">
-        <v>283</v>
+        <v>278</v>
+      </c>
+      <c r="B135" t="s">
+        <v>286</v>
       </c>
       <c r="C135">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D135">
         <v>1</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>278</v>
+        <v>18</v>
       </c>
       <c r="F135">
         <v>-1</v>
@@ -7276,19 +7264,19 @@
     </row>
     <row r="136" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>281</v>
-      </c>
-      <c r="B136" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
+      </c>
+      <c r="B136" t="s">
+        <v>287</v>
       </c>
       <c r="C136">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D136">
         <v>1</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>278</v>
+        <v>18</v>
       </c>
       <c r="F136">
         <v>-1</v>
@@ -7320,10 +7308,10 @@
     </row>
     <row r="137" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B137" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C137">
         <v>100</v>
@@ -7364,10 +7352,10 @@
     </row>
     <row r="138" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B138" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C138">
         <v>100</v>
@@ -7408,10 +7396,10 @@
     </row>
     <row r="139" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B139" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C139">
         <v>100</v>
@@ -7447,94 +7435,6 @@
         <v>0</v>
       </c>
       <c r="N139">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>288</v>
-      </c>
-      <c r="B140" t="s">
-        <v>293</v>
-      </c>
-      <c r="C140">
-        <v>100</v>
-      </c>
-      <c r="D140">
-        <v>1</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F140">
-        <v>-1</v>
-      </c>
-      <c r="G140">
-        <v>0</v>
-      </c>
-      <c r="H140">
-        <v>0</v>
-      </c>
-      <c r="I140">
-        <v>0</v>
-      </c>
-      <c r="J140">
-        <v>0</v>
-      </c>
-      <c r="K140">
-        <v>0</v>
-      </c>
-      <c r="L140">
-        <v>0</v>
-      </c>
-      <c r="M140">
-        <v>0</v>
-      </c>
-      <c r="N140">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>289</v>
-      </c>
-      <c r="B141" t="s">
-        <v>294</v>
-      </c>
-      <c r="C141">
-        <v>100</v>
-      </c>
-      <c r="D141">
-        <v>1</v>
-      </c>
-      <c r="E141" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F141">
-        <v>-1</v>
-      </c>
-      <c r="G141">
-        <v>0</v>
-      </c>
-      <c r="H141">
-        <v>0</v>
-      </c>
-      <c r="I141">
-        <v>0</v>
-      </c>
-      <c r="J141">
-        <v>0</v>
-      </c>
-      <c r="K141">
-        <v>0</v>
-      </c>
-      <c r="L141">
-        <v>0</v>
-      </c>
-      <c r="M141">
-        <v>0</v>
-      </c>
-      <c r="N141">
         <v>0</v>
       </c>
     </row>

</xml_diff>